<commit_message>
nabeel Traders STT Done
</commit_message>
<xml_diff>
--- a/Sep_2026/daily Reports/Daily Booking VS Execution.xlsx
+++ b/Sep_2026/daily Reports/Daily Booking VS Execution.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\786\Desktop\Elite-Git\Sep_2026\Daily Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8A75938-311A-4581-B77C-6D90E932A1A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{144BEC19-04E4-4E5A-AABD-94DC4F286434}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="860" activeTab="10" xr2:uid="{B0E336F2-AB38-4CE9-B7A3-449981D50C07}"/>
   </bookViews>
@@ -3188,7 +3188,7 @@
     <col min="18" max="18" width="3.08984375" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="3.90625" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="3.6328125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="3.08984375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="3.54296875" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="5.453125" customWidth="1"/>
     <col min="25" max="25" width="7.453125" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="9.36328125" bestFit="1" customWidth="1"/>
@@ -3814,17 +3814,31 @@
         <v>16</v>
       </c>
       <c r="O13" s="11"/>
-      <c r="P13" s="11"/>
-      <c r="Q13" s="11"/>
-      <c r="R13" s="11"/>
-      <c r="S13" s="11"/>
-      <c r="T13" s="11"/>
-      <c r="U13" s="11"/>
+      <c r="P13" s="11">
+        <v>240</v>
+      </c>
+      <c r="Q13" s="11">
+        <v>360</v>
+      </c>
+      <c r="R13" s="11">
+        <v>720</v>
+      </c>
+      <c r="S13" s="11">
+        <v>480</v>
+      </c>
+      <c r="T13" s="11">
+        <v>560</v>
+      </c>
+      <c r="U13" s="11">
+        <v>1200</v>
+      </c>
       <c r="V13" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="W13" s="12"/>
+        <v>89</v>
+      </c>
+      <c r="W13" s="12">
+        <v>4</v>
+      </c>
       <c r="Y13" s="36"/>
       <c r="Z13" s="37"/>
       <c r="AA13" s="38"/>
@@ -4031,31 +4045,31 @@
       </c>
       <c r="P18" s="25">
         <f t="shared" si="6"/>
-        <v>74</v>
+        <v>314</v>
       </c>
       <c r="Q18" s="25">
         <f t="shared" si="6"/>
-        <v>63</v>
+        <v>423</v>
       </c>
       <c r="R18" s="25">
         <f t="shared" si="6"/>
-        <v>64</v>
+        <v>784</v>
       </c>
       <c r="S18" s="25">
         <f t="shared" si="6"/>
-        <v>223</v>
+        <v>703</v>
       </c>
       <c r="T18" s="25">
         <f t="shared" si="6"/>
-        <v>154</v>
+        <v>714</v>
       </c>
       <c r="U18" s="25">
         <f t="shared" si="6"/>
-        <v>317</v>
+        <v>1517</v>
       </c>
       <c r="V18" s="26">
         <f>SUM(O18:U18)</f>
-        <v>1127</v>
+        <v>4687</v>
       </c>
       <c r="W18" s="28"/>
       <c r="Y18" s="33">
@@ -4119,31 +4133,31 @@
       </c>
       <c r="P19" s="21">
         <f t="shared" si="8"/>
-        <v>1.85</v>
+        <v>7.85</v>
       </c>
       <c r="Q19" s="21">
         <f t="shared" si="8"/>
-        <v>1.575</v>
+        <v>10.574999999999999</v>
       </c>
       <c r="R19" s="21">
         <f t="shared" si="8"/>
-        <v>1.6</v>
+        <v>19.600000000000001</v>
       </c>
       <c r="S19" s="21">
         <f t="shared" si="8"/>
-        <v>5.5750000000000002</v>
+        <v>17.574999999999999</v>
       </c>
       <c r="T19" s="21">
         <f t="shared" si="8"/>
-        <v>3.85</v>
+        <v>17.850000000000001</v>
       </c>
       <c r="U19" s="21">
         <f t="shared" si="8"/>
-        <v>7.9249999999999998</v>
+        <v>37.924999999999997</v>
       </c>
       <c r="V19" s="22">
         <f t="shared" si="8"/>
-        <v>28.175000000000001</v>
+        <v>117.175</v>
       </c>
       <c r="W19" s="23"/>
       <c r="Y19" s="39">

</xml_diff>